<commit_message>
image-hough with drawing hough line works, found most significant 7 hough lines
</commit_message>
<xml_diff>
--- a/src/320x240gray_sobel_orientation_0.bin.hough.xlsx
+++ b/src/320x240gray_sobel_orientation_0.bin.hough.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\Dropbox\software\projects\cv\cv-workbench\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B3ECD66A-144D-47E9-9177-1957CB4C7651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{0513E083-9905-41D6-8CEA-6C7A4A893915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576"/>
   </bookViews>
@@ -553,7 +553,14 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -571,7 +578,21 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFCC00FF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -596,8 +617,20 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFCC00FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -76288,17 +76321,23 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="between">
       <formula>35000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="between">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="between">
       <formula>25000</formula>
       <formula>30000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="between">
       <formula>20000</formula>
       <formula>25000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="DI21">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="between">
+      <formula>15000</formula>
+      <formula>20000</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>